<commit_message>
mindisp were missing new techs
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_advanced_features.xlsx
+++ b/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_advanced_features.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30E25BEB-3AD9-4047-893F-A421EDB16807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C6DB7F-B752-42A9-AFCB-B93B348F73E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="6" xr2:uid="{22AE2797-EE70-457C-AC96-4BB7B6BD4E04}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="278">
   <si>
     <t>ACT_MINLD</t>
   </si>
@@ -2843,9 +2843,6 @@
     <t>ELE,CHP</t>
   </si>
   <si>
-    <t>E*</t>
-  </si>
-  <si>
     <t>Min dispatchable capacity for VRE portfolio</t>
   </si>
   <si>
@@ -2861,7 +2858,7 @@
     <t>distr*</t>
   </si>
   <si>
-    <t>*,-solar,-wind*,-ELC,-ELCSPV,-elc[_]???[_]*</t>
+    <t>*,-solar,-wind*,-ELC,-ELCSPV,-elc[_]???[_]*,-e[_]*</t>
   </si>
 </sst>
 </file>
@@ -6807,7 +6804,7 @@
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C5" t="s">
         <v>252</v>
@@ -6818,7 +6815,7 @@
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C6" t="s">
         <v>254</v>
@@ -6829,7 +6826,7 @@
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C7" t="s">
         <v>255</v>
@@ -6893,11 +6890,8 @@
       <c r="C22" t="s">
         <v>271</v>
       </c>
-      <c r="D22" t="s">
-        <v>272</v>
-      </c>
       <c r="E22" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I22">
         <v>1</v>
@@ -6909,12 +6903,12 @@
         <v>5</v>
       </c>
       <c r="M22" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.45">
       <c r="G23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J23">
         <v>-1</v>

</xml_diff>